<commit_message>
Update dashboard and add key query output screenshots
</commit_message>
<xml_diff>
--- a/dashboard/ecommerce_dashboard.xlsx
+++ b/dashboard/ecommerce_dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/51dc9a68cc0015d2/Desktop/ecommerce-sales-analysis/dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="907" documentId="13_ncr:1_{A6188133-36C7-448F-81E9-FA1A37D88FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EB0104B-C085-4B62-83C0-5D56A416D7A1}"/>
+  <xr:revisionPtr revIDLastSave="911" documentId="13_ncr:1_{A6188133-36C7-448F-81E9-FA1A37D88FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{065DC6F4-44CB-4580-A60F-40357BD9B74A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="348" yWindow="744" windowWidth="14124" windowHeight="8928" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="monthly_revenue" sheetId="2" r:id="rId1"/>
@@ -16008,7 +16008,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
@@ -16202,16 +16202,16 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>160019</xdr:rowOff>
+      <xdr:rowOff>152400</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>34</xdr:row>
-      <xdr:rowOff>76200</xdr:rowOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>175260</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="6" name="product_category_name 1">
@@ -16234,7 +16234,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -16244,8 +16244,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="0" y="4914899"/>
-              <a:ext cx="1828800" cy="1562101"/>
+              <a:off x="0" y="4907280"/>
+              <a:ext cx="1828800" cy="1485900"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>

</xml_diff>